<commit_message>
`fix: import mockpass person ids for bulk student login`
</commit_message>
<xml_diff>
--- a/scripts/test-data/test-data-002-auto-lifecycle-bulk-import.xlsx
+++ b/scripts/test-data/test-data-002-auto-lifecycle-bulk-import.xlsx
@@ -166,72 +166,72 @@
         <t>Optional: Numeric school organization id. Optional when SchoolName is supplied or school can be resolved.</t>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <t>Required: Valid Singapore NRIC/FIN, including checksum. Example: S1234567D.</t>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <t>Required: Student full name, maximum 200 characters.</t>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
+    <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>Required: Use a real Excel date or yyyy-mm-dd. Student age must be 6 to 40 years.</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>Required: Nationality code, maximum 30 characters. Example: SG.</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>Optional: Citizenship code, maximum 30 characters. Example: CITIZEN.</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <t>Required: School student number, maximum 50 characters.</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>Required: Academic year text, maximum 20 characters. Example: 2026.</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="K1" authorId="0" shapeId="0">
       <text>
         <t>Required: Choose one: POST_SEC, BACHELOR, MASTER, PHD.</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <t>Optional: Class code, maximum 30 characters.</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <t>Optional: Use a real Excel date or yyyy-mm-dd. Must not be earlier than DateOfBirth.</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <t>Optional: Valid email address, maximum 320 characters.</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <t>Optional: Mobile/contact number, maximum 50 characters.</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <t>Optional: Residential address, maximum 1000 characters.</t>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <t>Keep SAMPLE_DO_NOT_IMPORT only on a sample row. Leave blank for real student data.</t>
       </text>
@@ -529,12 +529,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
@@ -561,72 +561,77 @@
           <t>OrganizationId</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MockPassPersonId</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>IdentityNumber</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>FullName</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>DateOfBirth</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>NationalityCode</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>CitizenshipStatusCode</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>StudentNumber</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>AcademicYear</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>LevelCode</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ClassCode</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>StartDate</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Mobile</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>TemplateRow</t>
         </is>
@@ -638,61 +643,66 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>9c9b5d05-1abd-4e11-817f-37c94f26be56</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>S7000029F</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Hannah Lim</t>
         </is>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="F2" s="4" t="n">
         <v>38092</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>QA-BULK001-001-SMU-2026-009</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>SMU-2026-009</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>POST_SEC</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>CLASS-POST_SEC-01</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="n">
+          <t>BACHELOR</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>SMU-Y1-03</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>bulk001.001.s7000029f@student.example.test</t>
-        </is>
-      </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>hannah.lim.smu009@student.example.test</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>+6591000029</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>29 Education Avenue, Singapore 100029</t>
         </is>
@@ -704,63 +714,68 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>S7000031H</t>
+          <t>bd68ebe6-8847-46d1-8774-0160e0c773d7</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Jia Min Lim</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>37166</v>
-      </c>
-      <c r="F3" t="inlineStr">
+          <t>S7000030G</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Isaac Lim</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>38555</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>QA-BULK001-002-SUTD-2026-001</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>SMU-2026-010</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>BACHELOR</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>CLASS-BACHELOR-02</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="n">
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>SMU-Y2-01</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>bulk001.002.s7000031h@student.example.test</t>
-        </is>
-      </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>+6591000031</t>
+          <t>isaac.lim.smu010@student.example.test</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>31 Education Avenue, Singapore 100031</t>
+          <t>+6591000030</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>30 Education Avenue, Singapore 100030</t>
         </is>
       </c>
     </row>
@@ -770,63 +785,68 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>S7000048B</t>
+          <t>b964c08b-a798-458c-bce0-46c306da1ab6</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Grace Lee</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>37634</v>
-      </c>
-      <c r="F4" t="inlineStr">
+          <t>S7000031H</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Jia Min Lim</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>37166</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>VALID_PASS_HOLDER</t>
-        </is>
-      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>QA-BULK001-003-SIT-2026-008</t>
+          <t>CITIZEN</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>SUTD-2026-001</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>MASTER</t>
-        </is>
-      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>CLASS-MASTER-03</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="n">
+          <t>BACHELOR</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>SUTD-Y1-01</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>bulk001.003.s7000048b@student.example.test</t>
-        </is>
-      </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>+6591000048</t>
+          <t>jia.min.lim.sutd001@student.example.test</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>48 Education Avenue, Singapore 100048</t>
+          <t>+6591000031</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>31 Education Avenue, Singapore 100031</t>
         </is>
       </c>
     </row>
@@ -836,63 +856,68 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>S7000050D</t>
+          <t>28e41f28-5c7a-4c3f-9f38-dd45393a2bbc</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Isaac Lee</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>38560</v>
-      </c>
-      <c r="F5" t="inlineStr">
+          <t>S7000032J</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Kai Lim</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>37265</v>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>QA-BULK001-004-SIT-2026-010</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>SUTD-2026-002</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>PHD</t>
-        </is>
-      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>CLASS-PHD-04</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="n">
+          <t>BACHELOR</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>SUTD-Y2-02</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>bulk001.004.s7000050d@student.example.test</t>
-        </is>
-      </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>+6591000050</t>
+          <t>kai.lim.sutd002@student.example.test</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>50 Education Avenue, Singapore 100050</t>
+          <t>+6591000032</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>32 Education Avenue, Singapore 100032</t>
         </is>
       </c>
     </row>
@@ -902,63 +927,68 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>S7000092Z</t>
+          <t>717dac1c-c021-420b-b660-b94d041d7e67</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>QA TEST DEMO004 Pranav Menon NTU</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>36799</v>
-      </c>
-      <c r="F6" t="inlineStr">
+          <t>S7000033K</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Liyana Lim</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>37727</v>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>QA-BULK001-005-NTU-2026-092</t>
-        </is>
-      </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>SUTD-2026-003</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>POST_SEC</t>
-        </is>
-      </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>CLASS-POST_SEC-05</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="n">
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>SUTD-Y3-03</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>bulk001.005.s7000092z@student.example.test</t>
-        </is>
-      </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>+6591000092</t>
+          <t>liyana.lim.sutd003@student.example.test</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>92 Education Avenue, Singapore 100092</t>
+          <t>+6591000033</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>33 Education Avenue, Singapore 100033</t>
         </is>
       </c>
     </row>
@@ -968,63 +998,68 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>S7000099G</t>
+          <t>d5ce54ea-c2ab-4d29-bd4b-6905ffba67e3</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>QA TEST DEMO004 Caleb Wong SUTD</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>34292</v>
-      </c>
-      <c r="F7" t="inlineStr">
+          <t>S7000034L</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Marcus Lim</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>38191</v>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>VALID_PASS_HOLDER</t>
-        </is>
-      </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>QA-BULK001-006-SUTD-2026-099</t>
+          <t>CITIZEN</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>SUTD-2026-004</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>BACHELOR</t>
-        </is>
-      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>CLASS-BACHELOR-06</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="n">
+          <t>PHD</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>SUTD-Y4-01</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>bulk001.006.s7000099g@student.example.test</t>
-        </is>
-      </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>+6591000099</t>
+          <t>marcus.lim.sutd004@student.example.test</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>99 Education Avenue, Singapore 100099</t>
+          <t>+6591000034</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>34 Education Avenue, Singapore 100034</t>
         </is>
       </c>
     </row>
@@ -1034,63 +1069,68 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>S8100006I</t>
+          <t>619e2335-7ff5-4884-abf7-929a2156f9b2</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>QA BULK001 Student 007</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>39675</v>
-      </c>
-      <c r="F8" t="inlineStr">
+          <t>S7000035M</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Nadia Lim</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>38628</v>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>QA-BULK001-007</t>
-        </is>
-      </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t>SUTD-2026-005</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>MASTER</t>
-        </is>
-      </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>CLASS-MASTER-07</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="n">
+          <t>BACHELOR</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>SUTD-Y1-02</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>qa.bulk001.007@student.example.test</t>
-        </is>
-      </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>+6592010007</t>
+          <t>nadia.lim.sutd005@student.example.test</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>7 QA Bulk Import 001 Avenue</t>
+          <t>+6591000035</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>35 Education Avenue, Singapore 100035</t>
         </is>
       </c>
     </row>
@@ -1100,63 +1140,68 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>S8100007G</t>
+          <t>76cd6639-f486-43b7-acf0-4ba34f72f961</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>QA BULK001 Student 008</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>36786</v>
-      </c>
-      <c r="F9" t="inlineStr">
+          <t>S7000036N</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Oliver Lim</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>36901</v>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>QA-BULK001-008</t>
-        </is>
-      </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>SUTD-2026-006</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>PHD</t>
-        </is>
-      </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>CLASS-PHD-08</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="n">
+          <t>BACHELOR</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>SUTD-Y2-03</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>qa.bulk001.008@student.example.test</t>
-        </is>
-      </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>+6592010008</t>
+          <t>oliver.lim.sutd006@student.example.test</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>8 QA Bulk Import 001 Avenue</t>
+          <t>+6591000036</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>36 Education Avenue, Singapore 100036</t>
         </is>
       </c>
     </row>
@@ -1166,63 +1211,68 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>S8100008E</t>
+          <t>4c357bdb-2382-4105-8349-c30ef28a5c0d</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>QA BULK001 Student 009</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>37183</v>
-      </c>
-      <c r="F10" t="inlineStr">
+          <t>S7000037P</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Priya Lim</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>37363</v>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>VALID_PASS_HOLDER</t>
-        </is>
-      </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>QA-BULK001-009</t>
+          <t>CITIZEN</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>SUTD-2026-007</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>POST_SEC</t>
-        </is>
-      </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>CLASS-POST_SEC-09</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="n">
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>SUTD-Y3-01</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>qa.bulk001.009@student.example.test</t>
-        </is>
-      </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>+6592010009</t>
+          <t>priya.lim.sutd007@student.example.test</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>9 QA Bulk Import 001 Avenue</t>
+          <t>+6591000037</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>37 Education Avenue, Singapore 100037</t>
         </is>
       </c>
     </row>
@@ -1232,63 +1282,68 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>S8100009C</t>
+          <t>c2974885-5c5f-4df5-8515-4ecb840e90db</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>QA BULK001 Student 010</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>37561</v>
-      </c>
-      <c r="F11" t="inlineStr">
+          <t>S7000038Q</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Ryan Lim</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>37826</v>
+      </c>
+      <c r="G11" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>QA-BULK001-010</t>
-        </is>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>SUTD-2026-008</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>BACHELOR</t>
-        </is>
-      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>CLASS-BACHELOR-10</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="n">
+          <t>PHD</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>SUTD-Y4-02</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>qa.bulk001.010@student.example.test</t>
-        </is>
-      </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>+6592010010</t>
+          <t>ryan.lim.sutd008@student.example.test</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>10 QA Bulk Import 001 Avenue</t>
+          <t>+6591000038</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>38 Education Avenue, Singapore 100038</t>
         </is>
       </c>
     </row>
@@ -1298,63 +1353,68 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>S8100010G</t>
+          <t>75a84c54-f406-42e0-96c7-769fdfe64c70</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>QA BULK001 Student 011</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>37958</v>
-      </c>
-      <c r="F12" t="inlineStr">
+          <t>S7000039R</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Siti Lim</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>38264</v>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>QA-BULK001-011</t>
-        </is>
-      </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>SUTD-2026-009</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>MASTER</t>
-        </is>
-      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>CLASS-MASTER-11</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="n">
+          <t>BACHELOR</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>SUTD-Y1-03</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>qa.bulk001.011@student.example.test</t>
-        </is>
-      </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>+6592010011</t>
+          <t>siti.lim.sutd009@student.example.test</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>11 QA Bulk Import 001 Avenue</t>
+          <t>+6591000039</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>39 Education Avenue, Singapore 100039</t>
         </is>
       </c>
     </row>
@@ -1364,63 +1424,68 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>S8100011E</t>
+          <t>8c751878-9c50-40ba-adba-e980605817a6</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>QA BULK001 Student 012</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>37991</v>
-      </c>
-      <c r="F13" t="inlineStr">
+          <t>S7000040T</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Wei Jie Lim</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>38363</v>
+      </c>
+      <c r="G13" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>VALID_PASS_HOLDER</t>
-        </is>
-      </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>QA-BULK001-012</t>
+          <t>CITIZEN</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
+          <t>SUTD-2026-010</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>PHD</t>
-        </is>
-      </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>CLASS-PHD-12</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="n">
+          <t>BACHELOR</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>SUTD-Y2-01</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>qa.bulk001.012@student.example.test</t>
-        </is>
-      </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>+6592010012</t>
+          <t>wei.jie.lim.sutd010@student.example.test</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>12 QA Bulk Import 001 Avenue</t>
+          <t>+6591000040</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>40 Education Avenue, Singapore 100040</t>
         </is>
       </c>
     </row>
@@ -1430,63 +1495,68 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>S8100012C</t>
+          <t>91ad0a28-92a0-47ac-a29c-e5cc07835697</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>QA BULK001 Student 013</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>38390</v>
-      </c>
-      <c r="F14" t="inlineStr">
+          <t>S7000041U</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Aarav Lee</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>36999</v>
+      </c>
+      <c r="G14" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>QA-BULK001-013</t>
-        </is>
-      </c>
       <c r="I14" t="inlineStr">
         <is>
+          <t>SIT-2026-001</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>POST_SEC</t>
-        </is>
-      </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>CLASS-POST_SEC-13</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="n">
+          <t>BACHELOR</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>SIT-Y1-01</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>qa.bulk001.013@student.example.test</t>
-        </is>
-      </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>+6592010013</t>
+          <t>aarav.lee.sit001@student.example.test</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>13 QA Bulk Import 001 Avenue</t>
+          <t>+6591000041</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>41 Education Avenue, Singapore 100041</t>
         </is>
       </c>
     </row>
@@ -1496,63 +1566,68 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>S8100013A</t>
+          <t>a453341a-96e6-422f-889c-474ee17f5cec</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>QA BULK001 Student 014</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>38785</v>
-      </c>
-      <c r="F15" t="inlineStr">
+          <t>S7000042V</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Aisha Lee</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>37462</v>
+      </c>
+      <c r="G15" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>QA-BULK001-014</t>
-        </is>
-      </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>SIT-2026-002</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>BACHELOR</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>CLASS-BACHELOR-14</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="n">
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>SIT-Y2-02</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>qa.bulk001.014@student.example.test</t>
-        </is>
-      </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>+6592010014</t>
+          <t>aisha.lee.sit002@student.example.test</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>14 QA Bulk Import 001 Avenue</t>
+          <t>+6591000042</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>42 Education Avenue, Singapore 100042</t>
         </is>
       </c>
     </row>
@@ -1562,63 +1637,68 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>S8100014Z</t>
+          <t>2125c836-da1d-4a2b-b26b-e22dd1b99b8a</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>QA BULK001 Student 015</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>39183</v>
-      </c>
-      <c r="F16" t="inlineStr">
+          <t>S7000043W</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Benjamin Lee</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>37899</v>
+      </c>
+      <c r="G16" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>VALID_PASS_HOLDER</t>
-        </is>
-      </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>QA-BULK001-015</t>
+          <t>CITIZEN</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
+          <t>SIT-2026-003</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>MASTER</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>CLASS-MASTER-15</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="n">
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>SIT-Y3-03</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>qa.bulk001.015@student.example.test</t>
-        </is>
-      </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>+6592010015</t>
+          <t>benjamin.lee.sit003@student.example.test</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>15 QA Bulk Import 001 Avenue</t>
+          <t>+6591000043</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>43 Education Avenue, Singapore 100043</t>
         </is>
       </c>
     </row>
@@ -1628,63 +1708,68 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>S8100015H</t>
+          <t>d5b8c485-4ab1-497b-a0bb-9feefcebde71</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>QA BULK001 Student 016</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>39581</v>
-      </c>
-      <c r="F17" t="inlineStr">
+          <t>S7000044X</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Chloe Lee</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>37998</v>
+      </c>
+      <c r="G17" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>QA-BULK001-016</t>
-        </is>
-      </c>
       <c r="I17" t="inlineStr">
         <is>
+          <t>SIT-2026-004</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>PHD</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>CLASS-PHD-16</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="n">
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>SIT-Y4-01</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>qa.bulk001.016@student.example.test</t>
-        </is>
-      </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>+6592010016</t>
+          <t>chloe.lee.sit004@student.example.test</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>16 QA Bulk Import 001 Avenue</t>
+          <t>+6591000044</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>44 Education Avenue, Singapore 100044</t>
         </is>
       </c>
     </row>
@@ -1694,63 +1779,68 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>S8100016F</t>
+          <t>8b49de77-611f-4897-bb44-e9ba90aa585d</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>QA BULK001 Student 017</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="n">
-        <v>36692</v>
-      </c>
-      <c r="F18" t="inlineStr">
+          <t>S7000045Y</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Daniel Lee</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>38461</v>
+      </c>
+      <c r="G18" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>QA-BULK001-017</t>
-        </is>
-      </c>
       <c r="I18" t="inlineStr">
         <is>
+          <t>SIT-2026-005</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>POST_SEC</t>
-        </is>
-      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>CLASS-POST_SEC-17</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="n">
+          <t>BACHELOR</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>SIT-Y1-02</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>qa.bulk001.017@student.example.test</t>
-        </is>
-      </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>+6592010017</t>
+          <t>daniel.lee.sit005@student.example.test</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>17 QA Bulk Import 001 Avenue</t>
+          <t>+6591000045</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>45 Education Avenue, Singapore 100045</t>
         </is>
       </c>
     </row>
@@ -1758,65 +1848,65 @@
       <c r="B19" t="n">
         <v>2</v>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>A7000029A</t>
-        </is>
-      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>QA BULK001 Invalid Checksum</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>38092</v>
-      </c>
-      <c r="F19" t="inlineStr">
+          <t>A7000046Z</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Emma Lee</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>37098</v>
+      </c>
+      <c r="G19" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>QA-BULK001-INVALID-NRIC</t>
-        </is>
-      </c>
       <c r="I19" t="inlineStr">
         <is>
+          <t>SIT-2026-006</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>POST_SEC</t>
-        </is>
-      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>CLASS-POST_SEC-01</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="n">
+          <t>BACHELOR</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>SIT-Y2-03</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>qa.bulk001.invalid.nric@student.example.test</t>
-        </is>
-      </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>+6591000029</t>
+          <t>emma.lee.sit006@student.example.test</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>29 Education Avenue, Singapore 100029</t>
+          <t>+6591000046</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>46 Education Avenue, Singapore 100046</t>
         </is>
       </c>
     </row>
@@ -1826,58 +1916,64 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>S8800001C</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>37166</v>
-      </c>
-      <c r="F20" t="inlineStr">
+          <t>61275942-e60f-4aa3-969b-a313e4c7ccc9</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>S7000046Z</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" s="4" t="n">
+        <v>37098</v>
+      </c>
+      <c r="G20" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>CITIZEN</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>QA-BULK001-MISSING-NAME</t>
-        </is>
-      </c>
       <c r="I20" t="inlineStr">
         <is>
+          <t>SIT-2026-006</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>BACHELOR</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>CLASS-BACHELOR-02</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="n">
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>SIT-Y2-03</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="n">
         <v>46024</v>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>qa.bulk001.missing.name@student.example.test</t>
-        </is>
-      </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>+6591000031</t>
+          <t>emma.lee.sit006@student.example.test</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>31 Education Avenue, Singapore 100031</t>
+          <t>+6591000046</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>46 Education Avenue, Singapore 100046</t>
         </is>
       </c>
     </row>
@@ -1887,63 +1983,68 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>S8900001G</t>
+          <t>796dca6f-69e2-481f-9b0c-bbeb158d9d92</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>QA BULK001 Invalid Start Date</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>39580</v>
-      </c>
-      <c r="F21" t="inlineStr">
+          <t>S7000047A</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Farhan Lee</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>37535</v>
+      </c>
+      <c r="G21" t="inlineStr">
         <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>VALID_PASS_HOLDER</t>
-        </is>
-      </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>QA-BULK001-BAD-START</t>
+          <t>CITIZEN</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
+          <t>SIT-2026-007</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>MASTER</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>CLASS-MASTER-03</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="n">
-        <v>39084</v>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>qa.bulk001.bad.start@student.example.test</t>
-        </is>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>SIT-Y3-01</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="n">
+        <v>37534</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>+6591000048</t>
+          <t>farhan.lee.sit007@student.example.test</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>48 Education Avenue, Singapore 100048</t>
+          <t>+6591000047</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>47 Education Avenue, Singapore 100047</t>
         </is>
       </c>
     </row>

</xml_diff>